<commit_message>
Migrate original Lines of Effort content into refined tracker
Populate the refined workbook with the seven Lines of Effort from the
original tracker, converting priority values (1 - Critical -> Critical),
deriving End State / Output entries where the existing row made them
unambiguous, and dropping the removed Staff Function, Category and Status
fields after confirming their useful content is preserved in Next Action
and Notes. Original dates retained, correctly surfacing all seven lines
as stale in the summary band.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FpsGqGN1EaS9r7pD8jv17k
</commit_message>
<xml_diff>
--- a/output/Lines of Effort Tracker - Refined.xlsx
+++ b/output/Lines of Effort Tracker - Refined.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="45">
   <si>
     <t xml:space="preserve">LINES OF EFFORT</t>
   </si>
@@ -68,19 +68,94 @@
     <t xml:space="preserve">LAST UPDATED</t>
   </si>
   <si>
+    <t xml:space="preserve">Critical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NZALC Operating Manual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manual approved, published and in use</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finalise critical incident chapter.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Core chapters drafted; final review pending.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Budget Builder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY26/27 budget model confirmed and issued</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirm FY26/27 figures and lock template.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model working; awaiting final figures.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY Summary Production Process</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Production process documented as a written SOP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Document final production steps.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Process mapped; needs written SOP.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Important</t>
   </si>
   <si>
-    <t xml:space="preserve">Example — replace with a Line of Effort</t>
+    <t xml:space="preserve">Course Nomination &amp; Preparation SOP</t>
   </si>
   <si>
     <t xml:space="preserve">SOP approved and implemented</t>
   </si>
   <si>
-    <t xml:space="preserve">Draft to XO for review</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Placeholder row — overwrite with real content</t>
+    <t xml:space="preserve">Review with Dave.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Draft complete; with reviewer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assistant Training Coordinator Proposal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proposal endorsed and responsibilities handed over</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prepare handover brief.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Case built; handover plan forming.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Storeperson Performance &amp; Workforce Assurance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resubmit establishment request.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Early stage; establishment case scoping.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Routine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Training Manager Job Evaluation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recommendation submitted for command decision</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Draft recommendation paper.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Queued behind priority items.</t>
   </si>
   <si>
     <t xml:space="preserve">Add new Lines of Effort in the first empty row — the table, dropdowns and formatting extend automatically.  Dates: dd mmm yy.  Stale = not updated in 14 days.</t>
@@ -335,7 +410,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="11">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -362,7 +437,31 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FF8A8781"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9E1B20"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FF3F3E3B"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFA87B2A"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -719,23 +818,23 @@
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="5" t="n">
         <f aca="false">COUNTA(C11:C400)</f>
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D7" s="5" t="n">
         <f aca="false">COUNTIF(B11:B400,"Critical")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">COUNTIF(B11:B400,"Important")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G7" s="5" t="n">
         <f aca="false">COUNTIF(B11:B400,"Routine")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H7" s="5" t="n">
         <f aca="true">COUNTIF(H11:H400,"&lt;"&amp;TODAY()-14)</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -763,7 +862,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="8" t="s">
         <v>14</v>
       </c>
@@ -774,7 +873,7 @@
         <v>16</v>
       </c>
       <c r="E11" s="11" t="n">
-        <v>0.45</v>
+        <v>0.8</v>
       </c>
       <c r="F11" s="10" t="s">
         <v>17</v>
@@ -783,62 +882,144 @@
         <v>18</v>
       </c>
       <c r="H11" s="13" t="n">
-        <v>46260</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="8"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="13"/>
-    </row>
-    <row r="13" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="8"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="13"/>
-    </row>
-    <row r="14" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="8"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="13"/>
-    </row>
-    <row r="15" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="8"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="13"/>
-    </row>
-    <row r="16" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="8"/>
-      <c r="C16" s="9"/>
+        <v>46181</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="H12" s="13" t="n">
+        <v>46181</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="G13" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="H13" s="13" t="n">
+        <v>46181</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="G14" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="H14" s="13" t="n">
+        <v>46181</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="G15" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="H15" s="13" t="n">
+        <v>46181</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>36</v>
+      </c>
       <c r="D16" s="10"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="13"/>
-    </row>
-    <row r="17" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="8"/>
-      <c r="C17" s="9"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="13"/>
+      <c r="E16" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="G16" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="H16" s="13" t="n">
+        <v>46181</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="G17" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="H17" s="13" t="n">
+        <v>46181</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="8"/>
@@ -905,25 +1086,25 @@
     </row>
     <row r="27" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="14" t="s">
-        <v>19</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="H7">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>$H$7&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11:B400">
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>$B11="Critical"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>$B11="Routine"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11:H400">
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>AND($H11&lt;&gt;"",$H11&lt;TODAY()-14)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -936,7 +1117,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{90B88024-4250-4BF4-B72C-D43ED5EBCE8E}</x14:id>
+          <x14:id>{C04EC47C-9AE9-4F73-8C48-5268DF951B26}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -965,7 +1146,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{90B88024-4250-4BF4-B72C-D43ED5EBCE8E}">
+          <x14:cfRule type="dataBar" id="{C04EC47C-9AE9-4F73-8C48-5268DF951B26}">
             <x14:dataBar minLength="0" maxLength="100" axisPosition="none" gradient="false" border="false">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>

<commit_message>
Add lines of effort arising from the AITC and course rationalisation meeting
Add five new lines: Junior Officer Leadership Training (Critical), TFCC
course correction and TF instructor transition, Alpine Touring resource
review, psychometric and workforce continuity (Important), and the 11 Oct
Civil Support session (Routine). Update ELDA Comd Review with the 5-day
package question from the same discussion. Row heights now size to their
content so longer end states and notes no longer clip.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FpsGqGN1EaS9r7pD8jv17k
</commit_message>
<xml_diff>
--- a/output/Lines of Effort Tracker - Refined.xlsx
+++ b/output/Lines of Effort Tracker - Refined.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="93">
   <si>
     <t xml:space="preserve">NZALC HQ - LINES OF EFFORT TRACKER</t>
   </si>
@@ -66,6 +66,18 @@
   </si>
   <si>
     <t xml:space="preserve">Critical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Junior Officer Leadership Training</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Foundational leadership intervention for junior officers formally endorsed through AITC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirm direction with the boss, then draft the 1–2 page proposition for early Sep AITC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tight scope — a training requirement, not the NZDF system. HQ ACS ownership. Courtesy comms to Sam/Cat/psych once agreed.</t>
   </si>
   <si>
     <t xml:space="preserve">Combat Mindset Submission</t>
@@ -186,6 +198,42 @@
     <t xml:space="preserve">Early/mid Nov (potential dates)</t>
   </si>
   <si>
+    <t xml:space="preserve">TFCC Course Correction &amp; TF Instructor Transition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Erroneous RF course requirement removed and TF instructor delivery in place</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Call Billy Vince to remove the RF course requirement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replace the requirement with the intended leadership outcomes. Instructor transition follows the December TTT. Phone, not email.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alpine Touring Resource Review</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resource model decided — reduced internal footprint, contractor support, or course ceased</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conduct the resource review with Tony</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Five staff plus significant preparation and gear for one annual course is difficult to justify.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Psychometric &amp; Workforce Continuity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">September staffing decisions confirmed with cover in place</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clarify the James option for off-site psychometric administration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Responsibilities don't align to national position descriptions. September is the decision point — keep HR engagement moving.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Routine</t>
   </si>
   <si>
@@ -237,16 +285,25 @@
     <t xml:space="preserve">Review completed and reported</t>
   </si>
   <si>
-    <t xml:space="preserve">No update at this stage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not yet started.</t>
+    <t xml:space="preserve">Determine whether the 8–10 day model can become a ~5-day package</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not yet started — progress figure needs correcting.</t>
   </si>
   <si>
     <t xml:space="preserve">Support to HUMINT Platoon FTX</t>
   </si>
   <si>
     <t xml:space="preserve">Support delivered to FTX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Civil Support Session (11 Oct 26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Session delivered with 360-focused instructor support</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calendar the session and allocate one — preferably two — instructors</t>
   </si>
 </sst>
 </file>
@@ -643,8 +700,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblLoE" displayName="tblLoE" ref="A7:G28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A7:G28"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblLoE" displayName="tblLoE" ref="A7:G33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A7:G33"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Priority"/>
     <tableColumn id="2" name="Line of Effort"/>
@@ -837,7 +894,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.5"/>
@@ -884,24 +941,24 @@
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="n">
         <f aca="false">COUNTA(B8:B41)</f>
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="5" t="n">
         <f aca="false">COUNTIF(A8:A41,"Critical")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D5" s="5" t="n">
         <f aca="false">COUNTIF(A8:A41,"Important")</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E5" s="5" t="n">
         <f aca="false">COUNTIF(A8:A41,"Routine")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F5" s="4" t="n">
         <f aca="true">COUNTIF(G8:G41,"&lt;"&amp;TODAY()-14)</f>
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G5" s="4"/>
     </row>
@@ -929,25 +986,27 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
         <v>13</v>
       </c>
       <c r="B8" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="9"/>
+      <c r="C8" s="9" t="s">
+        <v>15</v>
+      </c>
       <c r="D8" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>46244</v>
+        <v>46261</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -955,81 +1014,85 @@
         <v>13</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="9" t="s">
         <v>18</v>
       </c>
+      <c r="C9" s="9"/>
       <c r="D9" s="10" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E9" s="9"/>
+        <v>1</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>19</v>
+      </c>
       <c r="F9" s="9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G9" s="11" t="n">
         <v>46244</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
         <v>13</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D10" s="10" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="F10" s="9"/>
+        <v>0.6</v>
+      </c>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9" t="s">
+        <v>23</v>
+      </c>
       <c r="G10" s="11" t="n">
         <v>46244</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
         <v>13</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F11" s="9" t="s">
         <v>26</v>
       </c>
+      <c r="F11" s="9"/>
       <c r="G11" s="11" t="n">
         <v>46244</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
         <v>13</v>
       </c>
       <c r="B12" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="9"/>
+      <c r="C12" s="9" t="s">
+        <v>28</v>
+      </c>
       <c r="D12" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
+        <v>0.5</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>30</v>
+      </c>
       <c r="G12" s="11" t="n">
-        <v>46204</v>
+        <v>46244</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1037,7 +1100,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C13" s="9"/>
       <c r="D13" s="10" t="n">
@@ -1046,7 +1109,7 @@
       <c r="E13" s="9"/>
       <c r="F13" s="9"/>
       <c r="G13" s="11" t="n">
-        <v>46211</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1054,25 +1117,21 @@
         <v>13</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>30</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="C14" s="9"/>
       <c r="D14" s="10" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E14" s="9"/>
-      <c r="F14" s="9" t="s">
-        <v>31</v>
-      </c>
+      <c r="F14" s="9"/>
       <c r="G14" s="11" t="n">
-        <v>46244</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="B15" s="9" t="s">
         <v>33</v>
@@ -1081,21 +1140,19 @@
         <v>34</v>
       </c>
       <c r="D15" s="10" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E15" s="9" t="s">
+        <v>0.5</v>
+      </c>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9" t="s">
         <v>35</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>36</v>
       </c>
       <c r="G15" s="11" t="n">
         <v>46244</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B16" s="9" t="s">
         <v>37</v>
@@ -1104,7 +1161,7 @@
         <v>38</v>
       </c>
       <c r="D16" s="10" t="n">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="E16" s="9" t="s">
         <v>39</v>
@@ -1116,20 +1173,24 @@
         <v>46244</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B17" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C17" s="9"/>
+      <c r="C17" s="9" t="s">
+        <v>42</v>
+      </c>
       <c r="D17" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" s="9"/>
+        <v>0.7</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>43</v>
+      </c>
       <c r="F17" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G17" s="11" t="n">
         <v>46244</v>
@@ -1137,49 +1198,45 @@
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>44</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="C18" s="9"/>
       <c r="D18" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
+      <c r="F18" s="9" t="s">
+        <v>46</v>
+      </c>
       <c r="G18" s="11" t="n">
+        <v>46244</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="11" t="n">
         <v>46230</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="D19" s="10" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="F19" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="G19" s="11" t="n">
-        <v>46244</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B20" s="9" t="s">
         <v>49</v>
@@ -1188,7 +1245,7 @@
         <v>50</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="E20" s="9" t="s">
         <v>51</v>
@@ -1197,171 +1254,284 @@
         <v>52</v>
       </c>
       <c r="G20" s="11" t="n">
+        <v>46244</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D21" s="10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="G21" s="11" t="n">
         <v>46240</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="B21" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="C21" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="D21" s="10" t="n">
+    <row r="22" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="D22" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="11" t="n">
-        <v>46244</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="B22" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="C22" s="9"/>
-      <c r="D22" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
+      <c r="E22" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>60</v>
+      </c>
       <c r="G22" s="11" t="n">
-        <v>46244</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="D23" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="G23" s="11" t="n">
-        <v>46244</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="D24" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="9"/>
+        <v>0</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>67</v>
+      </c>
       <c r="F24" s="9" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="G24" s="11" t="n">
-        <v>46205</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
       <c r="G25" s="11" t="n">
-        <v>46230</v>
+        <v>46244</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C26" s="9" t="s">
-        <v>66</v>
-      </c>
+        <v>72</v>
+      </c>
+      <c r="C26" s="9"/>
       <c r="D26" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E26" s="9"/>
-      <c r="F26" s="9" t="s">
-        <v>67</v>
-      </c>
+      <c r="F26" s="9"/>
       <c r="G26" s="11" t="n">
-        <v>46230</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>46244</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="D27" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="G27" s="11" t="n">
-        <v>46230</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>46244</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="D28" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E28" s="9"/>
       <c r="F28" s="9" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="G28" s="11" t="n">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="D29" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="9"/>
+      <c r="F29" s="9"/>
+      <c r="G29" s="11" t="n">
         <v>46230</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="D30" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="9"/>
+      <c r="F30" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="G30" s="11" t="n">
+        <v>46230</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="D31" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="G31" s="11" t="n">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="C32" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="D32" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="9"/>
+      <c r="F32" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="G32" s="11" t="n">
+        <v>46230</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B33" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="D33" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="F33" s="9"/>
+      <c r="G33" s="11" t="n">
+        <v>46261</v>
       </c>
     </row>
   </sheetData>
@@ -1402,7 +1572,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BC89C539-82E6-4034-B97F-7B4F31F76199}</x14:id>
+          <x14:id>{2D93C78C-BF60-4E3A-A2BA-B058DB9082A2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -1431,7 +1601,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BC89C539-82E6-4034-B97F-7B4F31F76199}">
+          <x14:cfRule type="dataBar" id="{2D93C78C-BF60-4E3A-A2BA-B058DB9082A2}">
             <x14:dataBar minLength="0" maxLength="100" axisPosition="none" gradient="false" border="false">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>